<commit_message>
Deployed 80b66321 to development with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/development/Orchestration/assets/Orchestration-1.2.0-XFHL-3.0.0-mapping.xlsx
+++ b/development/Orchestration/assets/Orchestration-1.2.0-XFHL-3.0.0-mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iataonline-my.sharepoint.com/personal/lambertc_iata_org/Documents/ONE Record/31 CXML mapping/Release 3.2.0 docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iataonline-my.sharepoint.com/personal/lambertc_iata_org/Documents/ONE Record/31 CXML mapping/Ochestration 1.2.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{D8687063-E2B8-410F-9BB7-19FE8E9735AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9090E13-61C2-4272-A0D2-DD30F5CDDB97}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{D8687063-E2B8-410F-9BB7-19FE8E9735AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23EC8080-8617-4CA4-AFEC-4C1506DFBFE9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{409C4CA4-810D-446E-B907-D73C99948B9B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="145">
   <si>
     <t>XML Structure</t>
   </si>
@@ -491,6 +491,12 @@
   </si>
   <si>
     <t>Waybill#houseWaybills &gt; Waybill#externalReference -&gt; ExternalReference#documentName</t>
+  </si>
+  <si>
+    <t>Waybill#arrivalLocation#locationCode</t>
+  </si>
+  <si>
+    <t>Waybill#arrivalLocation#locationName</t>
   </si>
 </sst>
 </file>
@@ -563,7 +569,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -582,7 +588,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -592,7 +597,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -915,37 +919,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>42</v>
       </c>
     </row>
@@ -959,8 +963,7 @@
   <dimension ref="A1:N184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" style="8" customWidth="1"/>
-    <col min="2" max="8" width="4.5703125" customWidth="1"/>
+    <col min="1" max="8" width="4.5703125" customWidth="1"/>
     <col min="9" max="9" width="37.42578125" customWidth="1"/>
     <col min="10" max="11" width="9.140625" style="4"/>
     <col min="12" max="12" width="77.42578125" bestFit="1" customWidth="1"/>
@@ -1044,43 +1047,43 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
-      <c r="C6" s="8" t="s">
+      <c r="C6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
-      <c r="C7" s="8" t="s">
+      <c r="C7" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
-      <c r="C8" s="8" t="s">
+      <c r="C8" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
-      <c r="C9" s="8" t="s">
+      <c r="C9" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
-      <c r="C10" s="8" t="s">
+      <c r="C10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
-      <c r="C11" s="8" t="s">
+      <c r="C11" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
-      <c r="C12" s="8" t="s">
+      <c r="C12" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1093,7 +1096,7 @@
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
-      <c r="D14" s="8" t="s">
+      <c r="D14" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1112,7 +1115,7 @@
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
-      <c r="D17" s="8" t="s">
+      <c r="D17" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1134,7 +1137,7 @@
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
-      <c r="C21" s="8" t="s">
+      <c r="C21" t="s">
         <v>49</v>
       </c>
       <c r="I21" t="s">
@@ -1167,7 +1170,6 @@
         <v>83</v>
       </c>
       <c r="C23" s="1"/>
-      <c r="D23" s="8"/>
       <c r="J23" s="4" t="s">
         <v>19</v>
       </c>
@@ -1180,10 +1182,9 @@
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
-      <c r="C24" s="8" t="s">
+      <c r="C24" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="8"/>
       <c r="I24" t="s">
         <v>23</v>
       </c>
@@ -1202,7 +1203,7 @@
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
-      <c r="C25" s="8" t="s">
+      <c r="C25" t="s">
         <v>58</v>
       </c>
       <c r="I25" t="s">
@@ -1223,7 +1224,7 @@
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
-      <c r="C26" s="8" t="s">
+      <c r="C26" t="s">
         <v>59</v>
       </c>
       <c r="I26" t="s">
@@ -1244,7 +1245,7 @@
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
-      <c r="C27" s="8" t="s">
+      <c r="C27" t="s">
         <v>60</v>
       </c>
       <c r="I27" t="s">
@@ -1273,7 +1274,7 @@
     <row r="29" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
-      <c r="D29" s="8" t="s">
+      <c r="D29" t="s">
         <v>49</v>
       </c>
       <c r="I29" t="s">
@@ -1306,7 +1307,7 @@
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
-      <c r="D32" s="8" t="s">
+      <c r="D32" t="s">
         <v>49</v>
       </c>
       <c r="I32" t="s">
@@ -1325,7 +1326,7 @@
     <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
-      <c r="D33" s="8" t="s">
+      <c r="D33" t="s">
         <v>50</v>
       </c>
       <c r="I33" t="s">
@@ -1358,7 +1359,7 @@
     <row r="36" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
-      <c r="D36" s="8" t="s">
+      <c r="D36" t="s">
         <v>49</v>
       </c>
       <c r="I36" t="s">
@@ -1371,13 +1372,13 @@
         <v>20</v>
       </c>
       <c r="M36" t="s">
-        <v>117</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
-      <c r="D37" s="8" t="s">
+      <c r="D37" t="s">
         <v>50</v>
       </c>
       <c r="I37" t="s">
@@ -1390,7 +1391,7 @@
         <v>22</v>
       </c>
       <c r="M37" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
@@ -1398,7 +1399,6 @@
       <c r="C38" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D38" s="8"/>
       <c r="K38" s="6"/>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.25">
@@ -1411,7 +1411,7 @@
     <row r="40" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
-      <c r="D40" s="8" t="s">
+      <c r="D40" t="s">
         <v>61</v>
       </c>
       <c r="I40" t="s">
@@ -1430,10 +1430,9 @@
     <row r="41" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
-      <c r="D41" s="8" t="s">
+      <c r="D41" t="s">
         <v>62</v>
       </c>
-      <c r="E41" s="8"/>
       <c r="I41" t="s">
         <v>26</v>
       </c>
@@ -1450,7 +1449,7 @@
     <row r="42" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
-      <c r="D42" s="8" t="s">
+      <c r="D42" t="s">
         <v>63</v>
       </c>
       <c r="E42" s="1"/>
@@ -1470,7 +1469,7 @@
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
-      <c r="D43" s="8" t="s">
+      <c r="D43" t="s">
         <v>64</v>
       </c>
       <c r="E43" s="1"/>
@@ -1492,7 +1491,6 @@
       <c r="C44" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E44" s="8"/>
       <c r="K44" s="5"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.25">
@@ -1500,7 +1498,6 @@
       <c r="C45" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E45" s="8"/>
       <c r="J45" s="4" t="s">
         <v>19</v>
       </c>
@@ -1513,10 +1510,9 @@
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
-      <c r="D46" s="8" t="s">
+      <c r="D46" t="s">
         <v>65</v>
       </c>
-      <c r="E46" s="8"/>
       <c r="I46" t="s">
         <v>102</v>
       </c>
@@ -1532,7 +1528,7 @@
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
-      <c r="D47" s="8" t="s">
+      <c r="D47" t="s">
         <v>66</v>
       </c>
       <c r="I47" t="s">
@@ -1550,7 +1546,7 @@
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
-      <c r="D48" s="8" t="s">
+      <c r="D48" t="s">
         <v>59</v>
       </c>
       <c r="I48" t="s">
@@ -1568,7 +1564,7 @@
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
-      <c r="D49" s="8" t="s">
+      <c r="D49" t="s">
         <v>60</v>
       </c>
       <c r="E49" s="1"/>
@@ -1587,7 +1583,7 @@
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
-      <c r="D50" s="8" t="s">
+      <c r="D50" t="s">
         <v>67</v>
       </c>
       <c r="E50" s="1"/>
@@ -1615,7 +1611,7 @@
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
       <c r="D52" s="1"/>
-      <c r="E52" s="8" t="s">
+      <c r="E52" t="s">
         <v>49</v>
       </c>
       <c r="I52" t="s">
@@ -1648,7 +1644,7 @@
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
       <c r="D55" s="1"/>
-      <c r="E55" s="8" t="s">
+      <c r="E55" t="s">
         <v>49</v>
       </c>
       <c r="I55" t="s">
@@ -1667,7 +1663,7 @@
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
       <c r="D56" s="1"/>
-      <c r="E56" s="8" t="s">
+      <c r="E56" t="s">
         <v>50</v>
       </c>
       <c r="I56" t="s">
@@ -1700,7 +1696,7 @@
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
       <c r="D59" s="1"/>
-      <c r="E59" s="8" t="s">
+      <c r="E59" t="s">
         <v>49</v>
       </c>
       <c r="I59" t="s">
@@ -1719,7 +1715,7 @@
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
       <c r="D60" s="1"/>
-      <c r="E60" s="8" t="s">
+      <c r="E60" t="s">
         <v>50</v>
       </c>
       <c r="I60" t="s">
@@ -1752,7 +1748,7 @@
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
       <c r="D63" s="1"/>
-      <c r="E63" s="8" t="s">
+      <c r="E63" t="s">
         <v>68</v>
       </c>
       <c r="I63" t="s">
@@ -1771,7 +1767,7 @@
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
       <c r="D64" s="1"/>
-      <c r="E64" s="8" t="s">
+      <c r="E64" t="s">
         <v>69</v>
       </c>
       <c r="I64" t="s">
@@ -1800,7 +1796,7 @@
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="8" t="s">
+      <c r="E67" t="s">
         <v>68</v>
       </c>
       <c r="I67" t="s">
@@ -1819,7 +1815,7 @@
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
       <c r="D68" s="1"/>
-      <c r="E68" s="8" t="s">
+      <c r="E68" t="s">
         <v>69</v>
       </c>
       <c r="I68" t="s">
@@ -1837,7 +1833,6 @@
       <c r="D69" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E69" s="8"/>
       <c r="K69" s="6"/>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
@@ -1845,13 +1840,12 @@
       <c r="D70" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E70" s="8"/>
       <c r="K70" s="6"/>
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
       <c r="D71" s="1"/>
-      <c r="E71" s="8" t="s">
+      <c r="E71" t="s">
         <v>68</v>
       </c>
       <c r="I71" t="s">
@@ -1870,7 +1864,7 @@
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="8" t="s">
+      <c r="E72" t="s">
         <v>69</v>
       </c>
       <c r="I72" t="s">
@@ -1888,7 +1882,6 @@
       <c r="D73" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E73" s="8"/>
       <c r="K73" s="6"/>
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.25">
@@ -1896,13 +1889,12 @@
       <c r="D74" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E74" s="8"/>
       <c r="K74" s="5"/>
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
       <c r="D75" s="1"/>
-      <c r="E75" s="8" t="s">
+      <c r="E75" t="s">
         <v>61</v>
       </c>
       <c r="I75" t="s">
@@ -1921,7 +1913,7 @@
     <row r="76" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
       <c r="D76" s="1"/>
-      <c r="E76" s="8" t="s">
+      <c r="E76" t="s">
         <v>62</v>
       </c>
       <c r="I76" t="s">
@@ -1940,10 +1932,9 @@
     <row r="77" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
       <c r="D77" s="1"/>
-      <c r="E77" s="8" t="s">
+      <c r="E77" t="s">
         <v>63</v>
       </c>
-      <c r="F77" s="8"/>
       <c r="I77" t="s">
         <v>27</v>
       </c>
@@ -1960,7 +1951,7 @@
     <row r="78" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
       <c r="D78" s="1"/>
-      <c r="E78" s="8" t="s">
+      <c r="E78" t="s">
         <v>64</v>
       </c>
       <c r="I78" t="s">
@@ -1990,7 +1981,6 @@
         <v>88</v>
       </c>
       <c r="E80" s="1"/>
-      <c r="F80" s="8"/>
       <c r="J80" s="4" t="s">
         <v>21</v>
       </c>
@@ -2003,10 +1993,9 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
-      <c r="E81" s="8" t="s">
+      <c r="E81" t="s">
         <v>49</v>
       </c>
-      <c r="F81" s="8"/>
       <c r="I81" t="s">
         <v>106</v>
       </c>
@@ -2022,7 +2011,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
-      <c r="E82" s="8" t="s">
+      <c r="E82" t="s">
         <v>52</v>
       </c>
       <c r="I82" t="s">
@@ -2040,10 +2029,10 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
-      <c r="E83" s="8" t="s">
+      <c r="E83" t="s">
         <v>73</v>
       </c>
-      <c r="I83" s="12" t="s">
+      <c r="I83" t="s">
         <v>108</v>
       </c>
       <c r="J83" s="4" t="s">
@@ -2058,11 +2047,10 @@
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
-      <c r="E84" s="8" t="s">
+      <c r="E84" t="s">
         <v>50</v>
       </c>
-      <c r="F84" s="8"/>
-      <c r="I84" s="12" t="s">
+      <c r="I84" t="s">
         <v>109</v>
       </c>
       <c r="J84" s="4" t="s">
@@ -2080,7 +2068,6 @@
       <c r="D85" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F85" s="8"/>
       <c r="K85" s="6"/>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.25">
@@ -2103,11 +2090,9 @@
         <v>77</v>
       </c>
       <c r="B88" s="1"/>
-      <c r="F88" s="8"/>
       <c r="K88" s="5"/>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F89" s="8"/>
       <c r="K89" s="5"/>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.25">
@@ -2120,19 +2105,15 @@
       <c r="F91" s="1"/>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F92" s="8"/>
       <c r="K92" s="6"/>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F93" s="8"/>
       <c r="K93" s="5"/>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F94" s="8"/>
       <c r="K94" s="6"/>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F95" s="8"/>
       <c r="K95" s="6"/>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.25">
@@ -2143,7 +2124,6 @@
     </row>
     <row r="98" spans="5:11" x14ac:dyDescent="0.25">
       <c r="E98" s="1"/>
-      <c r="F98" s="8"/>
       <c r="K98" s="6"/>
     </row>
     <row r="99" spans="5:11" x14ac:dyDescent="0.25">
@@ -2156,11 +2136,9 @@
       <c r="F100" s="1"/>
     </row>
     <row r="101" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="F101" s="8"/>
       <c r="K101" s="5"/>
     </row>
     <row r="102" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="F102" s="8"/>
       <c r="K102" s="5"/>
     </row>
     <row r="103" spans="5:11" x14ac:dyDescent="0.25">
@@ -2168,15 +2146,12 @@
       <c r="K103" s="5"/>
     </row>
     <row r="104" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="G104" s="8"/>
       <c r="K104" s="5"/>
     </row>
     <row r="105" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="G105" s="8"/>
       <c r="K105" s="5"/>
     </row>
     <row r="106" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="G106" s="8"/>
       <c r="K106" s="5"/>
     </row>
     <row r="107" spans="5:11" x14ac:dyDescent="0.25">
@@ -2195,18 +2170,15 @@
       <c r="F109" s="1"/>
     </row>
     <row r="110" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="F110" s="8"/>
       <c r="K110" s="5"/>
     </row>
     <row r="111" spans="5:11" x14ac:dyDescent="0.25">
       <c r="F111" s="1"/>
     </row>
     <row r="112" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="G112" s="8"/>
       <c r="K112" s="5"/>
     </row>
     <row r="113" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="G113" s="8"/>
       <c r="K113" s="5"/>
     </row>
     <row r="114" spans="5:11" x14ac:dyDescent="0.25">
@@ -2222,11 +2194,9 @@
       <c r="K116" s="6"/>
     </row>
     <row r="117" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="H117" s="8"/>
       <c r="K117" s="6"/>
     </row>
     <row r="118" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="H118" s="8"/>
       <c r="K118" s="6"/>
     </row>
     <row r="119" spans="5:11" x14ac:dyDescent="0.25">
@@ -2242,7 +2212,6 @@
     </row>
     <row r="122" spans="5:11" x14ac:dyDescent="0.25">
       <c r="F122" s="1"/>
-      <c r="G122" s="8"/>
       <c r="K122" s="6"/>
     </row>
     <row r="123" spans="5:11" x14ac:dyDescent="0.25">
@@ -2256,23 +2225,18 @@
       <c r="K125" s="5"/>
     </row>
     <row r="126" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="F126" s="8"/>
       <c r="K126" s="6"/>
     </row>
     <row r="127" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="F127" s="8"/>
       <c r="K127" s="6"/>
     </row>
     <row r="128" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="F128" s="8"/>
       <c r="K128" s="5"/>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F129" s="8"/>
       <c r="K129" s="6"/>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F130" s="8"/>
       <c r="K130" s="5"/>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.25">
@@ -2280,7 +2244,6 @@
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F132" s="1"/>
-      <c r="G132" s="8"/>
       <c r="K132" s="5"/>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.25">
@@ -2550,15 +2513,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003BD9F489D8A3CB4CB4A9ED284A3FCA6E" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9f6f1c074eaefb361d518fe95996ab9d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0298a7ca-5e45-41ce-82dd-77fd4fe196fc" xmlns:ns3="cd402ee1-b2ab-4875-af71-19f72223aa0b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9118947706f37de36bda36ecf87158af" ns2:_="" ns3:_="">
     <xsd:import namespace="0298a7ca-5e45-41ce-82dd-77fd4fe196fc"/>
@@ -2781,6 +2735,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B130662-8EB9-4540-BC8F-0D1232647753}">
   <ds:schemaRefs>
@@ -2799,14 +2762,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F75F45A3-32E6-4084-931F-E62125045A6C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AB3A138-2C3A-40ED-BC06-2CB1DD202F66}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2825,6 +2780,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F75F45A3-32E6-4084-931F-E62125045A6C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{44ae014c-8170-484b-8a8e-3a6b842e2604}" enabled="1" method="Standard" siteId="{ad221784-72a8-4263-ac86-0ccc6b152cd8}" contentBits="1" removed="0"/>

</xml_diff>